<commit_message>
Add The Daily Heart and Paid in Full
The Daily Heart (Dr. Yusuf Al-Qalb, non-fiction) and Paid in Full (Yusuf Hasan,
fiction), with covers, descriptions and updated author intros.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GQVqzcb1uqdkAJ8RaWk7mn
</commit_message>
<xml_diff>
--- a/data/Final_Book_List.xlsx
+++ b/data/Final_Book_List.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E76"/>
+  <dimension ref="A1:E78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6.140625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -844,44 +844,44 @@
     </row>
     <row r="18">
       <c r="A18" s="4" t="n"/>
-      <c r="B18" s="4" t="n"/>
-      <c r="C18" s="4" t="n"/>
-      <c r="D18" s="4" t="n"/>
-      <c r="E18" s="4" t="n"/>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Dr. Yusuf Al-Qalb</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Non-fiction</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>The Daily Heart</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>https://mybook.to/dailyheart</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n"/>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t>Islamic Shia</t>
-        </is>
-      </c>
+      <c r="B19" s="4" t="n"/>
       <c r="C19" s="4" t="n"/>
       <c r="D19" s="4" t="n"/>
       <c r="E19" s="4" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n"/>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>Dr. Saiyed Ali Al-Razavi</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>Non-fiction</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>The Field of Karbala</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>https://mybook.to/FieldsofKarbala</t>
-        </is>
-      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Islamic Shia</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="n"/>
+      <c r="D20" s="4" t="n"/>
+      <c r="E20" s="4" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n"/>
@@ -897,12 +897,12 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Daughters of Revelation</t>
+          <t>The Field of Karbala</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>https://mybook.to/DaughtersOfRevelatio</t>
+          <t>https://mybook.to/FieldsofKarbala</t>
         </is>
       </c>
     </row>
@@ -920,12 +920,12 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Raising Shia Children in the West</t>
+          <t>Daughters of Revelation</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>https://mybook.to/RaisingShiaChildren</t>
+          <t>https://mybook.to/DaughtersOfRevelatio</t>
         </is>
       </c>
     </row>
@@ -943,12 +943,12 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Understanding the Twelve Imams</t>
+          <t>Raising Shia Children in the West</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>https://mybook.to/TwelveImams</t>
+          <t>https://mybook.to/RaisingShiaChildren</t>
         </is>
       </c>
     </row>
@@ -966,12 +966,12 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>The Shia Muslim Handbook</t>
+          <t>Understanding the Twelve Imams</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>https://mybook.to/ShiaMuslimHandbook</t>
+          <t>https://mybook.to/TwelveImams</t>
         </is>
       </c>
     </row>
@@ -989,12 +989,12 @@
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>The Next Marja</t>
+          <t>The Shia Muslim Handbook</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>https://mybook.to/Marja</t>
+          <t>https://mybook.to/ShiaMuslimHandbook</t>
         </is>
       </c>
     </row>
@@ -1012,12 +1012,12 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>The Shia Islam You've Heard About</t>
+          <t>The Next Marja</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>https://mybook.to/ShiaIslamHeardAbout</t>
+          <t>https://mybook.to/Marja</t>
         </is>
       </c>
     </row>
@@ -1035,12 +1035,12 @@
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Understanding the Shia</t>
+          <t>The Shia Islam You've Heard About</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>https://mybook.to/UnderstandingtheShia</t>
+          <t>https://mybook.to/ShiaIslamHeardAbout</t>
         </is>
       </c>
     </row>
@@ -1058,12 +1058,12 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Tears of the Ummah</t>
+          <t>Understanding the Shia</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>https://mybook.to/TearsoftheUmmah</t>
+          <t>https://mybook.to/UnderstandingtheShia</t>
         </is>
       </c>
     </row>
@@ -1081,55 +1081,55 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Whispers to the Divine</t>
+          <t>Tears of the Ummah</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>https://mybook.to/WhisperstotheDivine</t>
+          <t>https://mybook.to/TearsoftheUmmah</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n"/>
-      <c r="B30" s="4" t="n"/>
-      <c r="C30" s="4" t="n"/>
-      <c r="D30" s="4" t="n"/>
-      <c r="E30" s="4" t="n"/>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Dr. Saiyed Ali Al-Razavi</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Non-fiction</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>Whispers to the Divine</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>https://mybook.to/WhisperstotheDivine</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n"/>
-      <c r="B31" s="6" t="inlineStr">
-        <is>
-          <t>Self Mix</t>
-        </is>
-      </c>
+      <c r="B31" s="4" t="n"/>
       <c r="C31" s="4" t="n"/>
       <c r="D31" s="4" t="n"/>
       <c r="E31" s="4" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n"/>
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>Dr. Syed Ali Akbar Rizvi</t>
-        </is>
-      </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>Non-fiction</t>
-        </is>
-      </c>
-      <c r="D32" s="4" t="inlineStr">
-        <is>
-          <t>The Light of Divine Wisdom</t>
-        </is>
-      </c>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t>https://mybook.to/NahjulBalagha</t>
-        </is>
-      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>Self Mix</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="n"/>
+      <c r="D32" s="4" t="n"/>
+      <c r="E32" s="4" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n"/>
@@ -1145,12 +1145,12 @@
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Conversations with Allah the Al-Samīʿ</t>
+          <t>The Light of Divine Wisdom</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>https://mybook.to/ConversationsAllah</t>
+          <t>https://mybook.to/NahjulBalagha</t>
         </is>
       </c>
     </row>
@@ -1168,12 +1168,12 @@
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Shared Light</t>
+          <t>Conversations with Allah the Al-Samīʿ</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>https://mybook.to/SharedLight</t>
+          <t>https://mybook.to/ConversationsAllah</t>
         </is>
       </c>
     </row>
@@ -1186,17 +1186,17 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Fiction</t>
+          <t>Non-fiction</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>The 5 Intoxicants</t>
+          <t>Shared Light</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>https://mybook.to/5INTOXICANTS</t>
+          <t>https://mybook.to/SharedLight</t>
         </is>
       </c>
     </row>
@@ -1214,12 +1214,12 @@
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>The Lost and Found</t>
+          <t>The 5 Intoxicants</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>https://mybook.to/TheLostandFound</t>
+          <t>https://mybook.to/5INTOXICANTS</t>
         </is>
       </c>
     </row>
@@ -1237,55 +1237,55 @@
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Ninety Days More</t>
+          <t>The Lost and Found</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>https://mybook.to/90days</t>
+          <t>https://mybook.to/TheLostandFound</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="n"/>
-      <c r="B38" s="4" t="n"/>
-      <c r="C38" s="4" t="n"/>
-      <c r="D38" s="4" t="n"/>
-      <c r="E38" s="4" t="n"/>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Dr. Syed Ali Akbar Rizvi</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>Fiction</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>Ninety Days More</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>https://mybook.to/90days</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="n"/>
-      <c r="B39" s="6" t="inlineStr">
-        <is>
-          <t>Eleanor Hart</t>
-        </is>
-      </c>
+      <c r="B39" s="4" t="n"/>
       <c r="C39" s="4" t="n"/>
       <c r="D39" s="4" t="n"/>
       <c r="E39" s="4" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="n"/>
-      <c r="B40" s="4" t="inlineStr">
+      <c r="B40" s="6" t="inlineStr">
         <is>
           <t>Eleanor Hart</t>
         </is>
       </c>
-      <c r="C40" s="4" t="inlineStr">
-        <is>
-          <t>Fiction</t>
-        </is>
-      </c>
-      <c r="D40" s="4" t="inlineStr">
-        <is>
-          <t>The Ordinary Infinite</t>
-        </is>
-      </c>
-      <c r="E40" s="7" t="inlineStr">
-        <is>
-          <t>https://mybook.to/ORDINARYINFINITE</t>
-        </is>
-      </c>
+      <c r="C40" s="4" t="n"/>
+      <c r="D40" s="4" t="n"/>
+      <c r="E40" s="4" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="n"/>
@@ -1301,12 +1301,12 @@
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>All the Distance Between</t>
+          <t>The Ordinary Infinite</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t>https://mybook.to/DistanceBetween</t>
+          <t>https://mybook.to/ORDINARYINFINITE</t>
         </is>
       </c>
     </row>
@@ -1324,12 +1324,12 @@
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Weight of Light</t>
+          <t>All the Distance Between</t>
         </is>
       </c>
       <c r="E42" s="7" t="inlineStr">
         <is>
-          <t>https://mybook.to/WeightofLight</t>
+          <t>https://mybook.to/DistanceBetween</t>
         </is>
       </c>
     </row>
@@ -1347,12 +1347,12 @@
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>Almost</t>
+          <t>Weight of Light</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>https://mybook.to/AlmostNovel</t>
+          <t>https://mybook.to/WeightofLight</t>
         </is>
       </c>
     </row>
@@ -1365,101 +1365,101 @@
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Non-fiction</t>
+          <t>Fiction</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Estranged by Choice</t>
+          <t>Almost</t>
         </is>
       </c>
       <c r="E44" s="7" t="inlineStr">
         <is>
-          <t>https://mybook.to/EstrangedbyChoice</t>
+          <t>https://mybook.to/AlmostNovel</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="n"/>
-      <c r="B45" s="4" t="n"/>
-      <c r="C45" s="4" t="n"/>
-      <c r="D45" s="4" t="n"/>
-      <c r="E45" s="4" t="n"/>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>Eleanor Hart</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>Non-fiction</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>Estranged by Choice</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>https://mybook.to/EstrangedbyChoice</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="n"/>
-      <c r="B46" s="6" t="inlineStr">
-        <is>
-          <t>James Whitfield</t>
-        </is>
-      </c>
+      <c r="B46" s="4" t="n"/>
       <c r="C46" s="4" t="n"/>
       <c r="D46" s="4" t="n"/>
       <c r="E46" s="4" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="n"/>
-      <c r="B47" s="4" t="inlineStr">
+      <c r="B47" s="6" t="inlineStr">
         <is>
           <t>James Whitfield</t>
         </is>
       </c>
-      <c r="C47" s="4" t="inlineStr">
-        <is>
-          <t>Non-fiction</t>
-        </is>
-      </c>
-      <c r="D47" s="4" t="inlineStr">
-        <is>
-          <t>Still Standing: Keep Your Job</t>
-        </is>
-      </c>
-      <c r="E47" s="7" t="inlineStr">
-        <is>
-          <t>https://mybook.to/StillStandingAI</t>
-        </is>
-      </c>
+      <c r="C47" s="4" t="n"/>
+      <c r="D47" s="4" t="n"/>
+      <c r="E47" s="4" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="4" t="n"/>
-      <c r="B48" s="4" t="n"/>
-      <c r="C48" s="4" t="n"/>
-      <c r="D48" s="4" t="n"/>
-      <c r="E48" s="4" t="n"/>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>James Whitfield</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>Non-fiction</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>Still Standing: Keep Your Job</t>
+        </is>
+      </c>
+      <c r="E48" s="7" t="inlineStr">
+        <is>
+          <t>https://mybook.to/StillStandingAI</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="n"/>
-      <c r="B49" s="6" t="inlineStr">
-        <is>
-          <t>Julian Vale</t>
-        </is>
-      </c>
+      <c r="B49" s="4" t="n"/>
       <c r="C49" s="4" t="n"/>
       <c r="D49" s="4" t="n"/>
       <c r="E49" s="4" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="4" t="n"/>
-      <c r="B50" s="4" t="inlineStr">
+      <c r="B50" s="6" t="inlineStr">
         <is>
           <t>Julian Vale</t>
         </is>
       </c>
-      <c r="C50" s="4" t="inlineStr">
-        <is>
-          <t>Fiction</t>
-        </is>
-      </c>
-      <c r="D50" s="4" t="inlineStr">
-        <is>
-          <t>The Island of Second Chances</t>
-        </is>
-      </c>
-      <c r="E50" s="7" t="inlineStr">
-        <is>
-          <t>https://mybook.to/IslandofSecondChances</t>
-        </is>
-      </c>
+      <c r="C50" s="4" t="n"/>
+      <c r="D50" s="4" t="n"/>
+      <c r="E50" s="4" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="4" t="n"/>
@@ -1475,12 +1475,12 @@
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>The Last Train Before Morning</t>
+          <t>The Island of Second Chances</t>
         </is>
       </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>https://mybook.to/LastTrainBefore</t>
+          <t>https://mybook.to/IslandofSecondChances</t>
         </is>
       </c>
     </row>
@@ -1498,12 +1498,12 @@
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>The Ferryman</t>
+          <t>The Last Train Before Morning</t>
         </is>
       </c>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t>https://mybook.to/Ferryman</t>
+          <t>https://mybook.to/LastTrainBefore</t>
         </is>
       </c>
     </row>
@@ -1521,12 +1521,12 @@
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>The Gardener of Forgotten Dreams</t>
+          <t>The Ferryman</t>
         </is>
       </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t>https://mybook.to/TheGardenerDreams</t>
+          <t>https://mybook.to/Ferryman</t>
         </is>
       </c>
     </row>
@@ -1544,12 +1544,12 @@
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>The Shop That Sold Lost Things</t>
+          <t>The Gardener of Forgotten Dreams</t>
         </is>
       </c>
       <c r="E54" s="7" t="inlineStr">
         <is>
-          <t>https://mybook.to/LostThings</t>
+          <t>https://mybook.to/TheGardenerDreams</t>
         </is>
       </c>
     </row>
@@ -1567,12 +1567,12 @@
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>The Library of Unwritten Lives</t>
+          <t>The Shop That Sold Lost Things</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>https://mybook.to/UnwrittenLives</t>
+          <t>https://mybook.to/LostThings</t>
         </is>
       </c>
     </row>
@@ -1590,12 +1590,12 @@
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>The Man Who Collected Tomorrows</t>
+          <t>The Library of Unwritten Lives</t>
         </is>
       </c>
       <c r="E56" s="7" t="inlineStr">
         <is>
-          <t>https://mybook.to/CollectedTomorrows</t>
+          <t>https://mybook.to/UnwrittenLives</t>
         </is>
       </c>
     </row>
@@ -1613,12 +1613,12 @@
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>The Man Who Gave Away His Name</t>
-        </is>
-      </c>
-      <c r="E57" s="4" t="inlineStr">
-        <is>
-          <t>https://mybook.to/gaveawayname</t>
+          <t>The Man Who Collected Tomorrows</t>
+        </is>
+      </c>
+      <c r="E57" s="7" t="inlineStr">
+        <is>
+          <t>https://mybook.to/CollectedTomorrows</t>
         </is>
       </c>
     </row>
@@ -1636,12 +1636,12 @@
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>The House With Seven Doors</t>
+          <t>The Man Who Gave Away His Name</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>https://mybook.to/sevendoors</t>
+          <t>https://mybook.to/gaveawayname</t>
         </is>
       </c>
     </row>
@@ -1659,12 +1659,12 @@
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>The Castle at the End of the Road</t>
+          <t>The House With Seven Doors</t>
         </is>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t>https://mybook.to/Castleendofroad</t>
+          <t>https://mybook.to/sevendoors</t>
         </is>
       </c>
     </row>
@@ -1682,12 +1682,12 @@
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>The Garden Across the Street</t>
+          <t>The Castle at the End of the Road</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t>https://mybook.to/gardenacross</t>
+          <t>https://mybook.to/Castleendofroad</t>
         </is>
       </c>
     </row>
@@ -1705,12 +1705,12 @@
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>The Clockmaker Who Stopped Time</t>
+          <t>The Garden Across the Street</t>
         </is>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>https://mybook.to/clockmaker</t>
+          <t>https://mybook.to/gardenacross</t>
         </is>
       </c>
     </row>
@@ -1728,55 +1728,55 @@
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>The Uncollected</t>
+          <t>The Clockmaker Who Stopped Time</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>https://mybook.to/Uncollected</t>
+          <t>https://mybook.to/clockmaker</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="n"/>
-      <c r="B63" s="4" t="n"/>
-      <c r="C63" s="4" t="n"/>
-      <c r="D63" s="4" t="n"/>
-      <c r="E63" s="4" t="n"/>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>Julian Vale</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>Fiction</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>The Uncollected</t>
+        </is>
+      </c>
+      <c r="E63" s="4" t="inlineStr">
+        <is>
+          <t>https://mybook.to/Uncollected</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="n"/>
-      <c r="B64" s="6" t="inlineStr">
-        <is>
-          <t>Sage Norden, PhD</t>
-        </is>
-      </c>
+      <c r="B64" s="4" t="n"/>
       <c r="C64" s="4" t="n"/>
       <c r="D64" s="4" t="n"/>
       <c r="E64" s="4" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="4" t="n"/>
-      <c r="B65" s="4" t="inlineStr">
+      <c r="B65" s="6" t="inlineStr">
         <is>
           <t>Sage Norden, PhD</t>
         </is>
       </c>
-      <c r="C65" s="4" t="inlineStr">
-        <is>
-          <t>Non-fiction</t>
-        </is>
-      </c>
-      <c r="D65" s="4" t="inlineStr">
-        <is>
-          <t>The Jobs We Blamed on Machines</t>
-        </is>
-      </c>
-      <c r="E65" s="7" t="inlineStr">
-        <is>
-          <t>https://mybook.to/JobsweBlamed</t>
-        </is>
-      </c>
+      <c r="C65" s="4" t="n"/>
+      <c r="D65" s="4" t="n"/>
+      <c r="E65" s="4" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="4" t="n"/>
@@ -1792,12 +1792,12 @@
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>The Ally We Never Question</t>
+          <t>The Jobs We Blamed on Machines</t>
         </is>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>https://mybook.to/TheAlly</t>
+          <t>https://mybook.to/JobsweBlamed</t>
         </is>
       </c>
     </row>
@@ -1815,12 +1815,12 @@
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>The Governments We Unmade</t>
+          <t>The Ally We Never Question</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>https://mybook.to/GovernmentsWeUnmade</t>
+          <t>https://mybook.to/TheAlly</t>
         </is>
       </c>
     </row>
@@ -1838,12 +1838,12 @@
       </c>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t>The Dictators We Love</t>
+          <t>The Governments We Unmade</t>
         </is>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>https://mybook.to/DictatorsWeLove</t>
+          <t>https://mybook.to/GovernmentsWeUnmade</t>
         </is>
       </c>
     </row>
@@ -1861,12 +1861,12 @@
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>The Country That Stopped Learning</t>
+          <t>The Dictators We Love</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>https://mybook.to/COUNTRYTHATSTOPPED</t>
+          <t>https://mybook.to/DictatorsWeLove</t>
         </is>
       </c>
     </row>
@@ -1884,12 +1884,12 @@
       </c>
       <c r="D70" s="4" t="inlineStr">
         <is>
-          <t>Owned</t>
+          <t>The Country That Stopped Learning</t>
         </is>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>https://mybook.to/SurveillanceEconomy</t>
+          <t>https://mybook.to/COUNTRYTHATSTOPPED</t>
         </is>
       </c>
     </row>
@@ -1907,55 +1907,55 @@
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>The Comfort Tax</t>
+          <t>Owned</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr">
         <is>
-          <t>https://mybook.to/ComfortTax</t>
+          <t>https://mybook.to/SurveillanceEconomy</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="4" t="n"/>
-      <c r="B72" s="4" t="n"/>
-      <c r="C72" s="4" t="n"/>
-      <c r="D72" s="4" t="n"/>
-      <c r="E72" s="4" t="n"/>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>Sage Norden, PhD</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="inlineStr">
+        <is>
+          <t>Non-fiction</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t>The Comfort Tax</t>
+        </is>
+      </c>
+      <c r="E72" s="7" t="inlineStr">
+        <is>
+          <t>https://mybook.to/ComfortTax</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="n"/>
-      <c r="B73" s="6" t="inlineStr">
-        <is>
-          <t>Yusuf Hasan</t>
-        </is>
-      </c>
+      <c r="B73" s="4" t="n"/>
       <c r="C73" s="4" t="n"/>
       <c r="D73" s="4" t="n"/>
       <c r="E73" s="4" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="4" t="n"/>
-      <c r="B74" s="4" t="inlineStr">
+      <c r="B74" s="6" t="inlineStr">
         <is>
           <t>Yusuf Hasan</t>
         </is>
       </c>
-      <c r="C74" s="4" t="inlineStr">
-        <is>
-          <t>Fiction</t>
-        </is>
-      </c>
-      <c r="D74" s="4" t="inlineStr">
-        <is>
-          <t>Any Other Business</t>
-        </is>
-      </c>
-      <c r="E74" s="7" t="inlineStr">
-        <is>
-          <t>https://mybook.to/AnyOtherBusiness</t>
-        </is>
-      </c>
+      <c r="C74" s="4" t="n"/>
+      <c r="D74" s="4" t="n"/>
+      <c r="E74" s="4" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="4" t="n"/>
@@ -1971,12 +1971,12 @@
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>The Empty Cab</t>
+          <t>Any Other Business</t>
         </is>
       </c>
       <c r="E75" s="7" t="inlineStr">
         <is>
-          <t>https://mybook.to/THEEMPTYCAB</t>
+          <t>https://mybook.to/AnyOtherBusiness</t>
         </is>
       </c>
     </row>
@@ -1994,12 +1994,58 @@
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
+          <t>The Empty Cab</t>
+        </is>
+      </c>
+      <c r="E76" s="7" t="inlineStr">
+        <is>
+          <t>https://mybook.to/THEEMPTYCAB</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="n"/>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>Yusuf Hasan</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>Fiction</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="inlineStr">
+        <is>
           <t>The Fare</t>
         </is>
       </c>
-      <c r="E76" s="7" t="inlineStr">
+      <c r="E77" s="7" t="inlineStr">
         <is>
           <t>https://mybook.to/THEFARE</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="n"/>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>Yusuf Hasan</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t>Fiction</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t>Paid in Full</t>
+        </is>
+      </c>
+      <c r="E78" s="7" t="inlineStr">
+        <is>
+          <t>https://mybook.to/PaidinFull</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add The Other Chair by Julian Vale
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GQVqzcb1uqdkAJ8RaWk7mn
</commit_message>
<xml_diff>
--- a/data/Final_Book_List.xlsx
+++ b/data/Final_Book_List.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E78"/>
+  <dimension ref="A1:E79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6.140625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1285,7 +1285,11 @@
       </c>
       <c r="C40" s="4" t="n"/>
       <c r="D40" s="4" t="n"/>
-      <c r="E40" s="4" t="n"/>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>https://mybook.to/ORDINARYINFINITE</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="n"/>
@@ -1418,7 +1422,11 @@
       </c>
       <c r="C47" s="4" t="n"/>
       <c r="D47" s="4" t="n"/>
-      <c r="E47" s="4" t="n"/>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>https://mybook.to/StillStandingAI</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="n"/>
@@ -1459,7 +1467,11 @@
       </c>
       <c r="C50" s="4" t="n"/>
       <c r="D50" s="4" t="n"/>
-      <c r="E50" s="4" t="n"/>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>https://mybook.to/IslandofSecondChances</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="n"/>
@@ -1762,40 +1774,44 @@
     </row>
     <row r="64">
       <c r="A64" s="4" t="n"/>
-      <c r="B64" s="4" t="n"/>
-      <c r="C64" s="4" t="n"/>
-      <c r="D64" s="4" t="n"/>
-      <c r="E64" s="4" t="n"/>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t>Julian Vale</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t>Fiction</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>The Other Chair</t>
+        </is>
+      </c>
+      <c r="E64" s="4" t="inlineStr">
+        <is>
+          <t>https://mybook.to/TheOtherChair</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="n"/>
-      <c r="B65" s="6" t="inlineStr">
-        <is>
-          <t>Sage Norden, PhD</t>
-        </is>
-      </c>
+      <c r="B65" s="4" t="n"/>
       <c r="C65" s="4" t="n"/>
       <c r="D65" s="4" t="n"/>
       <c r="E65" s="4" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="4" t="n"/>
-      <c r="B66" s="4" t="inlineStr">
+      <c r="B66" s="6" t="inlineStr">
         <is>
           <t>Sage Norden, PhD</t>
         </is>
       </c>
-      <c r="C66" s="4" t="inlineStr">
-        <is>
-          <t>Non-fiction</t>
-        </is>
-      </c>
-      <c r="D66" s="4" t="inlineStr">
-        <is>
-          <t>The Jobs We Blamed on Machines</t>
-        </is>
-      </c>
-      <c r="E66" s="7" t="inlineStr">
+      <c r="C66" s="4" t="n"/>
+      <c r="D66" s="4" t="n"/>
+      <c r="E66" s="4" t="inlineStr">
         <is>
           <t>https://mybook.to/JobsweBlamed</t>
         </is>
@@ -1815,12 +1831,12 @@
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>The Ally We Never Question</t>
+          <t>The Jobs We Blamed on Machines</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>https://mybook.to/TheAlly</t>
+          <t>https://mybook.to/JobsweBlamed</t>
         </is>
       </c>
     </row>
@@ -1838,12 +1854,12 @@
       </c>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t>The Governments We Unmade</t>
+          <t>The Ally We Never Question</t>
         </is>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>https://mybook.to/GovernmentsWeUnmade</t>
+          <t>https://mybook.to/TheAlly</t>
         </is>
       </c>
     </row>
@@ -1861,12 +1877,12 @@
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>The Dictators We Love</t>
+          <t>The Governments We Unmade</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>https://mybook.to/DictatorsWeLove</t>
+          <t>https://mybook.to/GovernmentsWeUnmade</t>
         </is>
       </c>
     </row>
@@ -1884,12 +1900,12 @@
       </c>
       <c r="D70" s="4" t="inlineStr">
         <is>
-          <t>The Country That Stopped Learning</t>
+          <t>The Dictators We Love</t>
         </is>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>https://mybook.to/COUNTRYTHATSTOPPED</t>
+          <t>https://mybook.to/DictatorsWeLove</t>
         </is>
       </c>
     </row>
@@ -1907,12 +1923,12 @@
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>Owned</t>
+          <t>The Country That Stopped Learning</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr">
         <is>
-          <t>https://mybook.to/SurveillanceEconomy</t>
+          <t>https://mybook.to/COUNTRYTHATSTOPPED</t>
         </is>
       </c>
     </row>
@@ -1930,51 +1946,55 @@
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>The Comfort Tax</t>
+          <t>Owned</t>
         </is>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
-          <t>https://mybook.to/ComfortTax</t>
+          <t>https://mybook.to/SurveillanceEconomy</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="n"/>
-      <c r="B73" s="4" t="n"/>
-      <c r="C73" s="4" t="n"/>
-      <c r="D73" s="4" t="n"/>
-      <c r="E73" s="4" t="n"/>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>Sage Norden, PhD</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>Non-fiction</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t>The Comfort Tax</t>
+        </is>
+      </c>
+      <c r="E73" s="7" t="inlineStr">
+        <is>
+          <t>https://mybook.to/ComfortTax</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="4" t="n"/>
-      <c r="B74" s="6" t="inlineStr">
-        <is>
-          <t>Yusuf Hasan</t>
-        </is>
-      </c>
+      <c r="B74" s="4" t="n"/>
       <c r="C74" s="4" t="n"/>
       <c r="D74" s="4" t="n"/>
       <c r="E74" s="4" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="4" t="n"/>
-      <c r="B75" s="4" t="inlineStr">
+      <c r="B75" s="6" t="inlineStr">
         <is>
           <t>Yusuf Hasan</t>
         </is>
       </c>
-      <c r="C75" s="4" t="inlineStr">
-        <is>
-          <t>Fiction</t>
-        </is>
-      </c>
-      <c r="D75" s="4" t="inlineStr">
-        <is>
-          <t>Any Other Business</t>
-        </is>
-      </c>
-      <c r="E75" s="7" t="inlineStr">
+      <c r="C75" s="4" t="n"/>
+      <c r="D75" s="4" t="n"/>
+      <c r="E75" s="4" t="inlineStr">
         <is>
           <t>https://mybook.to/AnyOtherBusiness</t>
         </is>
@@ -1994,12 +2014,12 @@
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
-          <t>The Empty Cab</t>
+          <t>Any Other Business</t>
         </is>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>https://mybook.to/THEEMPTYCAB</t>
+          <t>https://mybook.to/AnyOtherBusiness</t>
         </is>
       </c>
     </row>
@@ -2017,12 +2037,12 @@
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>The Fare</t>
+          <t>The Empty Cab</t>
         </is>
       </c>
       <c r="E77" s="7" t="inlineStr">
         <is>
-          <t>https://mybook.to/THEFARE</t>
+          <t>https://mybook.to/THEEMPTYCAB</t>
         </is>
       </c>
     </row>
@@ -2040,10 +2060,33 @@
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
+          <t>The Fare</t>
+        </is>
+      </c>
+      <c r="E78" s="7" t="inlineStr">
+        <is>
+          <t>https://mybook.to/THEFARE</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="n"/>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>Yusuf Hasan</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="inlineStr">
+        <is>
+          <t>Fiction</t>
+        </is>
+      </c>
+      <c r="D79" s="4" t="inlineStr">
+        <is>
           <t>Paid in Full</t>
         </is>
       </c>
-      <c r="E78" s="7" t="inlineStr">
+      <c r="E79" s="7" t="inlineStr">
         <is>
           <t>https://mybook.to/PaidinFull</t>
         </is>

</xml_diff>

<commit_message>
Add Sorry, We're Open by Yusuf Hasan
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GQVqzcb1uqdkAJ8RaWk7mn
</commit_message>
<xml_diff>
--- a/data/Final_Book_List.xlsx
+++ b/data/Final_Book_List.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E79"/>
+  <dimension ref="A1:E80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6.140625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1800,7 +1800,11 @@
       <c r="B65" s="4" t="n"/>
       <c r="C65" s="4" t="n"/>
       <c r="D65" s="4" t="n"/>
-      <c r="E65" s="4" t="n"/>
+      <c r="E65" s="4" t="inlineStr">
+        <is>
+          <t>https://mybook.to/JobsweBlamed</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="4" t="n"/>
@@ -1983,7 +1987,11 @@
       <c r="B74" s="4" t="n"/>
       <c r="C74" s="4" t="n"/>
       <c r="D74" s="4" t="n"/>
-      <c r="E74" s="4" t="n"/>
+      <c r="E74" s="4" t="inlineStr">
+        <is>
+          <t>https://mybook.to/AnyOtherBusiness</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="n"/>
@@ -2089,6 +2097,29 @@
       <c r="E79" s="7" t="inlineStr">
         <is>
           <t>https://mybook.to/PaidinFull</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="n"/>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>Yusuf Hasan</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="inlineStr">
+        <is>
+          <t>Fiction</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="inlineStr">
+        <is>
+          <t>Sorry, We're Open</t>
+        </is>
+      </c>
+      <c r="E80" s="7" t="inlineStr">
+        <is>
+          <t>https://mybook.to/SorryOpen</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add authors Dev Malhotra and Anna Wray with their books
The Trouble with Us (non-fiction) and The Patient Who Never Lied (fiction,
Dr Claire Shaw series, Book 1), with covers.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GQVqzcb1uqdkAJ8RaWk7mn
</commit_message>
<xml_diff>
--- a/data/Final_Book_List.xlsx
+++ b/data/Final_Book_List.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E80"/>
+  <dimension ref="A1:E84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6.140625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -2120,6 +2120,52 @@
       <c r="E80" s="7" t="inlineStr">
         <is>
           <t>https://mybook.to/SorryOpen</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="n"/>
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t>Dev Malhotra</t>
+        </is>
+      </c>
+      <c r="C82" s="4" t="inlineStr">
+        <is>
+          <t>Non-fiction</t>
+        </is>
+      </c>
+      <c r="D82" s="4" t="inlineStr">
+        <is>
+          <t>The Trouble with Us</t>
+        </is>
+      </c>
+      <c r="E82" s="7" t="inlineStr">
+        <is>
+          <t>https://mybook.to/troublewithus</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="n"/>
+      <c r="B84" s="4" t="inlineStr">
+        <is>
+          <t>Anna Wray</t>
+        </is>
+      </c>
+      <c r="C84" s="4" t="inlineStr">
+        <is>
+          <t>Fiction</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>The Patient Who Never Lied</t>
+        </is>
+      </c>
+      <c r="E84" s="7" t="inlineStr">
+        <is>
+          <t>https://mybook.to/NeverLied</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add The Good Husband and What the Patient Knew by Anna Wray
Dr Claire Shaw series Books 2 and 3, with covers.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GQVqzcb1uqdkAJ8RaWk7mn
</commit_message>
<xml_diff>
--- a/data/Final_Book_List.xlsx
+++ b/data/Final_Book_List.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E84"/>
+  <dimension ref="A1:E86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6.140625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -2123,6 +2123,7 @@
         </is>
       </c>
     </row>
+    <row r="81"/>
     <row r="82">
       <c r="A82" s="4" t="n"/>
       <c r="B82" s="4" t="inlineStr">
@@ -2146,6 +2147,7 @@
         </is>
       </c>
     </row>
+    <row r="83"/>
     <row r="84">
       <c r="A84" s="4" t="n"/>
       <c r="B84" s="4" t="inlineStr">
@@ -2166,6 +2168,52 @@
       <c r="E84" s="7" t="inlineStr">
         <is>
           <t>https://mybook.to/NeverLied</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="n"/>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>Anna Wray</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="inlineStr">
+        <is>
+          <t>Fiction</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="inlineStr">
+        <is>
+          <t>The Good Husband</t>
+        </is>
+      </c>
+      <c r="E85" s="7" t="inlineStr">
+        <is>
+          <t>https://mybook.to/GoodHusband</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="n"/>
+      <c r="B86" s="4" t="inlineStr">
+        <is>
+          <t>Anna Wray</t>
+        </is>
+      </c>
+      <c r="C86" s="4" t="inlineStr">
+        <is>
+          <t>Fiction</t>
+        </is>
+      </c>
+      <c r="D86" s="4" t="inlineStr">
+        <is>
+          <t>What the Patient Knew</t>
+        </is>
+      </c>
+      <c r="E86" s="7" t="inlineStr">
+        <is>
+          <t>https://mybook.to/PatientKnew</t>
         </is>
       </c>
     </row>

</xml_diff>